<commit_message>
Fix number alignment across all documents
- index.html: ML metrics card updated (Propensity 0.73→0.78, LTV R²0.81→0.95, Churn→Cart Abandon 0.78→0.74)
- ebook.html: Stale SVG comments corrected to match live figures
- generate_excel.py: MONTHLY_REVENUE rebuilt — revenue now sums to $891,480, sessions to 1,891,200, transactions to 34,890; AOV varies by year ($25.23/$24.88/$26.39) matching YoY data in data.js
- GA4_Intelligence_Hub_Professional_v2.xlsx: regenerated with corrected Monthly Revenue sheet
</commit_message>
<xml_diff>
--- a/GA4_Intelligence_Hub_Professional_v2.xlsx
+++ b/GA4_Intelligence_Hub_Professional_v2.xlsx
@@ -14719,16 +14719,16 @@
         </is>
       </c>
       <c r="D3" s="67" t="n">
-        <v>18240</v>
+        <v>25180</v>
       </c>
       <c r="E3" s="68" t="n">
-        <v>14320</v>
+        <v>54090</v>
       </c>
       <c r="F3" s="68" t="n">
-        <v>714</v>
+        <v>998</v>
       </c>
       <c r="G3" s="69" t="n">
-        <v>25.55</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
@@ -14744,16 +14744,16 @@
         </is>
       </c>
       <c r="D4" s="67" t="n">
-        <v>47120</v>
+        <v>39586</v>
       </c>
       <c r="E4" s="68" t="n">
-        <v>37020</v>
+        <v>85000</v>
       </c>
       <c r="F4" s="68" t="n">
-        <v>1844</v>
+        <v>1569</v>
       </c>
       <c r="G4" s="69" t="n">
-        <v>25.55</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -14769,16 +14769,16 @@
         </is>
       </c>
       <c r="D5" s="73" t="n">
-        <v>22890</v>
+        <v>14028</v>
       </c>
       <c r="E5" s="74" t="n">
-        <v>17990</v>
+        <v>30140</v>
       </c>
       <c r="F5" s="74" t="n">
-        <v>896</v>
+        <v>556</v>
       </c>
       <c r="G5" s="75" t="n">
-        <v>25.55</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -14794,16 +14794,16 @@
         </is>
       </c>
       <c r="D6" s="73" t="n">
-        <v>19650</v>
+        <v>12413</v>
       </c>
       <c r="E6" s="74" t="n">
-        <v>15440</v>
+        <v>26660</v>
       </c>
       <c r="F6" s="74" t="n">
-        <v>769</v>
+        <v>492</v>
       </c>
       <c r="G6" s="75" t="n">
-        <v>25.55</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -14819,16 +14819,16 @@
         </is>
       </c>
       <c r="D7" s="73" t="n">
-        <v>23410</v>
+        <v>14936</v>
       </c>
       <c r="E7" s="74" t="n">
-        <v>18390</v>
+        <v>32070</v>
       </c>
       <c r="F7" s="74" t="n">
-        <v>916</v>
+        <v>592</v>
       </c>
       <c r="G7" s="75" t="n">
-        <v>25.55</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -14844,16 +14844,16 @@
         </is>
       </c>
       <c r="D8" s="73" t="n">
-        <v>21780</v>
+        <v>13498</v>
       </c>
       <c r="E8" s="74" t="n">
-        <v>17110</v>
+        <v>28980</v>
       </c>
       <c r="F8" s="74" t="n">
-        <v>852</v>
+        <v>535</v>
       </c>
       <c r="G8" s="75" t="n">
-        <v>25.55</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -14869,16 +14869,16 @@
         </is>
       </c>
       <c r="D9" s="73" t="n">
-        <v>24560</v>
+        <v>15643</v>
       </c>
       <c r="E9" s="74" t="n">
-        <v>19300</v>
+        <v>33620</v>
       </c>
       <c r="F9" s="74" t="n">
-        <v>961</v>
+        <v>620</v>
       </c>
       <c r="G9" s="75" t="n">
-        <v>25.55</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -14894,16 +14894,16 @@
         </is>
       </c>
       <c r="D10" s="73" t="n">
-        <v>22340</v>
+        <v>14381</v>
       </c>
       <c r="E10" s="74" t="n">
-        <v>17550</v>
+        <v>30910</v>
       </c>
       <c r="F10" s="74" t="n">
-        <v>874</v>
+        <v>570</v>
       </c>
       <c r="G10" s="75" t="n">
-        <v>25.55</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -14919,16 +14919,16 @@
         </is>
       </c>
       <c r="D11" s="73" t="n">
-        <v>20980</v>
+        <v>13498</v>
       </c>
       <c r="E11" s="74" t="n">
-        <v>16480</v>
+        <v>28980</v>
       </c>
       <c r="F11" s="74" t="n">
-        <v>821</v>
+        <v>535</v>
       </c>
       <c r="G11" s="75" t="n">
-        <v>25.55</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -14944,16 +14944,16 @@
         </is>
       </c>
       <c r="D12" s="73" t="n">
-        <v>25670</v>
+        <v>16551</v>
       </c>
       <c r="E12" s="74" t="n">
-        <v>20160</v>
+        <v>35550</v>
       </c>
       <c r="F12" s="74" t="n">
-        <v>1004</v>
+        <v>656</v>
       </c>
       <c r="G12" s="75" t="n">
-        <v>25.55</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
@@ -14969,16 +14969,16 @@
         </is>
       </c>
       <c r="D13" s="73" t="n">
-        <v>23890</v>
+        <v>15113</v>
       </c>
       <c r="E13" s="74" t="n">
-        <v>18770</v>
+        <v>32460</v>
       </c>
       <c r="F13" s="74" t="n">
-        <v>935</v>
+        <v>599</v>
       </c>
       <c r="G13" s="75" t="n">
-        <v>25.55</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -14994,16 +14994,16 @@
         </is>
       </c>
       <c r="D14" s="73" t="n">
-        <v>22110</v>
+        <v>13913</v>
       </c>
       <c r="E14" s="74" t="n">
-        <v>17380</v>
+        <v>29740</v>
       </c>
       <c r="F14" s="74" t="n">
-        <v>865</v>
+        <v>550</v>
       </c>
       <c r="G14" s="75" t="n">
-        <v>25.55</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -15019,16 +15019,16 @@
         </is>
       </c>
       <c r="D15" s="73" t="n">
-        <v>28290</v>
+        <v>39385</v>
       </c>
       <c r="E15" s="74" t="n">
-        <v>22220</v>
+        <v>83950</v>
       </c>
       <c r="F15" s="74" t="n">
-        <v>1107</v>
+        <v>1583</v>
       </c>
       <c r="G15" s="75" t="n">
-        <v>25.55</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -15044,16 +15044,16 @@
         </is>
       </c>
       <c r="D16" s="73" t="n">
-        <v>73060</v>
+        <v>61901</v>
       </c>
       <c r="E16" s="74" t="n">
-        <v>57380</v>
+        <v>131920</v>
       </c>
       <c r="F16" s="74" t="n">
-        <v>2859</v>
+        <v>2488</v>
       </c>
       <c r="G16" s="75" t="n">
-        <v>25.55</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -15069,16 +15069,16 @@
         </is>
       </c>
       <c r="D17" s="79" t="n">
-        <v>35480</v>
+        <v>21944</v>
       </c>
       <c r="E17" s="80" t="n">
-        <v>27870</v>
+        <v>46770</v>
       </c>
       <c r="F17" s="80" t="n">
-        <v>1388</v>
+        <v>882</v>
       </c>
       <c r="G17" s="81" t="n">
-        <v>25.55</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
@@ -15094,16 +15094,16 @@
         </is>
       </c>
       <c r="D18" s="79" t="n">
-        <v>30450</v>
+        <v>19406</v>
       </c>
       <c r="E18" s="80" t="n">
-        <v>23920</v>
+        <v>41380</v>
       </c>
       <c r="F18" s="80" t="n">
-        <v>1191</v>
+        <v>780</v>
       </c>
       <c r="G18" s="81" t="n">
-        <v>25.55</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -15119,16 +15119,16 @@
         </is>
       </c>
       <c r="D19" s="79" t="n">
-        <v>36270</v>
+        <v>23362</v>
       </c>
       <c r="E19" s="80" t="n">
-        <v>28490</v>
+        <v>49770</v>
       </c>
       <c r="F19" s="80" t="n">
-        <v>1419</v>
+        <v>939</v>
       </c>
       <c r="G19" s="81" t="n">
-        <v>25.55</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -15144,16 +15144,16 @@
         </is>
       </c>
       <c r="D20" s="79" t="n">
-        <v>33740</v>
+        <v>21098</v>
       </c>
       <c r="E20" s="80" t="n">
-        <v>26510</v>
+        <v>44970</v>
       </c>
       <c r="F20" s="80" t="n">
-        <v>1320</v>
+        <v>848</v>
       </c>
       <c r="G20" s="81" t="n">
-        <v>25.55</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
@@ -15169,16 +15169,16 @@
         </is>
       </c>
       <c r="D21" s="79" t="n">
-        <v>38070</v>
+        <v>24482</v>
       </c>
       <c r="E21" s="80" t="n">
-        <v>29920</v>
+        <v>52170</v>
       </c>
       <c r="F21" s="80" t="n">
-        <v>1490</v>
+        <v>984</v>
       </c>
       <c r="G21" s="81" t="n">
-        <v>25.55</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -15194,16 +15194,16 @@
         </is>
       </c>
       <c r="D22" s="79" t="n">
-        <v>34630</v>
+        <v>22516</v>
       </c>
       <c r="E22" s="80" t="n">
-        <v>27210</v>
+        <v>47970</v>
       </c>
       <c r="F22" s="80" t="n">
-        <v>1355</v>
+        <v>905</v>
       </c>
       <c r="G22" s="81" t="n">
-        <v>25.55</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -15219,16 +15219,16 @@
         </is>
       </c>
       <c r="D23" s="79" t="n">
-        <v>32520</v>
+        <v>21098</v>
       </c>
       <c r="E23" s="80" t="n">
-        <v>25550</v>
+        <v>44970</v>
       </c>
       <c r="F23" s="80" t="n">
-        <v>1272</v>
+        <v>848</v>
       </c>
       <c r="G23" s="81" t="n">
-        <v>25.55</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
@@ -15244,16 +15244,16 @@
         </is>
       </c>
       <c r="D24" s="79" t="n">
-        <v>39790</v>
+        <v>25900</v>
       </c>
       <c r="E24" s="80" t="n">
-        <v>31250</v>
+        <v>55170</v>
       </c>
       <c r="F24" s="80" t="n">
-        <v>1557</v>
+        <v>1041</v>
       </c>
       <c r="G24" s="81" t="n">
-        <v>25.55</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -15269,16 +15269,16 @@
         </is>
       </c>
       <c r="D25" s="79" t="n">
-        <v>37030</v>
+        <v>23636</v>
       </c>
       <c r="E25" s="80" t="n">
-        <v>29100</v>
+        <v>50370</v>
       </c>
       <c r="F25" s="80" t="n">
-        <v>1449</v>
+        <v>950</v>
       </c>
       <c r="G25" s="81" t="n">
-        <v>25.55</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -15294,16 +15294,16 @@
         </is>
       </c>
       <c r="D26" s="79" t="n">
-        <v>34280</v>
+        <v>21752</v>
       </c>
       <c r="E26" s="80" t="n">
-        <v>26930</v>
+        <v>46190</v>
       </c>
       <c r="F26" s="80" t="n">
-        <v>1341</v>
+        <v>872</v>
       </c>
       <c r="G26" s="81" t="n">
-        <v>25.55</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
@@ -15319,16 +15319,16 @@
         </is>
       </c>
       <c r="D27" s="79" t="n">
-        <v>43850</v>
+        <v>42989</v>
       </c>
       <c r="E27" s="80" t="n">
-        <v>34450</v>
+        <v>90200</v>
       </c>
       <c r="F27" s="80" t="n">
-        <v>1715</v>
+        <v>1629</v>
       </c>
       <c r="G27" s="81" t="n">
-        <v>25.55</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
@@ -15344,16 +15344,16 @@
         </is>
       </c>
       <c r="D28" s="79" t="n">
-        <v>113240</v>
+        <v>67558</v>
       </c>
       <c r="E28" s="80" t="n">
-        <v>88960</v>
+        <v>141750</v>
       </c>
       <c r="F28" s="80" t="n">
-        <v>4430</v>
+        <v>2560</v>
       </c>
       <c r="G28" s="81" t="n">
-        <v>25.55</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
@@ -15369,16 +15369,16 @@
         </is>
       </c>
       <c r="D29" s="85" t="n">
-        <v>38140</v>
+        <v>23962</v>
       </c>
       <c r="E29" s="86" t="n">
-        <v>29970</v>
+        <v>50260</v>
       </c>
       <c r="F29" s="86" t="n">
-        <v>1493</v>
+        <v>908</v>
       </c>
       <c r="G29" s="87" t="n">
-        <v>25.55</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
@@ -15394,16 +15394,16 @@
         </is>
       </c>
       <c r="D30" s="85" t="n">
-        <v>32740</v>
+        <v>21191</v>
       </c>
       <c r="E30" s="86" t="n">
-        <v>25720</v>
+        <v>44460</v>
       </c>
       <c r="F30" s="86" t="n">
-        <v>1281</v>
+        <v>803</v>
       </c>
       <c r="G30" s="87" t="n">
-        <v>25.55</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
@@ -15419,16 +15419,16 @@
         </is>
       </c>
       <c r="D31" s="85" t="n">
-        <v>39000</v>
+        <v>25493</v>
       </c>
       <c r="E31" s="86" t="n">
-        <v>30640</v>
+        <v>53480</v>
       </c>
       <c r="F31" s="86" t="n">
-        <v>1526</v>
+        <v>966</v>
       </c>
       <c r="G31" s="87" t="n">
-        <v>25.55</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
@@ -15444,16 +15444,16 @@
         </is>
       </c>
       <c r="D32" s="85" t="n">
-        <v>36270</v>
+        <v>23038</v>
       </c>
       <c r="E32" s="86" t="n">
-        <v>28490</v>
+        <v>48320</v>
       </c>
       <c r="F32" s="86" t="n">
-        <v>1419</v>
+        <v>873</v>
       </c>
       <c r="G32" s="87" t="n">
-        <v>25.55</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
@@ -15469,16 +15469,16 @@
         </is>
       </c>
       <c r="D33" s="85" t="n">
-        <v>40940</v>
+        <v>26707</v>
       </c>
       <c r="E33" s="86" t="n">
-        <v>32170</v>
+        <v>56060</v>
       </c>
       <c r="F33" s="86" t="n">
-        <v>1602</v>
+        <v>1012</v>
       </c>
       <c r="G33" s="87" t="n">
-        <v>25.55</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
@@ -15494,16 +15494,16 @@
         </is>
       </c>
       <c r="D34" s="85" t="n">
-        <v>37240</v>
+        <v>24569</v>
       </c>
       <c r="E34" s="86" t="n">
-        <v>29260</v>
+        <v>51540</v>
       </c>
       <c r="F34" s="86" t="n">
-        <v>1457</v>
+        <v>931</v>
       </c>
       <c r="G34" s="87" t="n">
-        <v>25.55</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
@@ -15519,16 +15519,16 @@
         </is>
       </c>
       <c r="D35" s="85" t="n">
-        <v>34960</v>
+        <v>23038</v>
       </c>
       <c r="E35" s="86" t="n">
-        <v>27470</v>
+        <v>48320</v>
       </c>
       <c r="F35" s="86" t="n">
-        <v>1368</v>
+        <v>873</v>
       </c>
       <c r="G35" s="87" t="n">
-        <v>25.55</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
@@ -15544,16 +15544,16 @@
         </is>
       </c>
       <c r="D36" s="85" t="n">
-        <v>42780</v>
+        <v>28264</v>
       </c>
       <c r="E36" s="86" t="n">
-        <v>33610</v>
+        <v>59280</v>
       </c>
       <c r="F36" s="86" t="n">
-        <v>1674</v>
+        <v>1071</v>
       </c>
       <c r="G36" s="87" t="n">
-        <v>25.55</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
@@ -15569,16 +15569,16 @@
         </is>
       </c>
       <c r="D37" s="85" t="n">
-        <v>39830</v>
+        <v>25783</v>
       </c>
       <c r="E37" s="86" t="n">
-        <v>31290</v>
+        <v>54120</v>
       </c>
       <c r="F37" s="86" t="n">
-        <v>1558</v>
+        <v>977</v>
       </c>
       <c r="G37" s="87" t="n">
-        <v>25.55</v>
+        <v>26.39</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
@@ -15594,16 +15594,16 @@
         </is>
       </c>
       <c r="D38" s="85" t="n">
-        <v>36860</v>
+        <v>23668</v>
       </c>
       <c r="E38" s="86" t="n">
-        <v>28970</v>
+        <v>49610</v>
       </c>
       <c r="F38" s="86" t="n">
-        <v>1442</v>
+        <v>895</v>
       </c>
       <c r="G38" s="87" t="n">
-        <v>25.55</v>
+        <v>26.39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>